<commit_message>
feat: add filter-config-service with CRUD operations for filter schema
- Implemented a new service for managing filter configurations, including endpoints for listing, creating, updating, and deleting filter schemas.
- Added database schema and connection handling using psycopg.
- Introduced seed data for initial filter configurations.
- Created a Dockerfile for containerization of the service.
- Added CORS support for cross-origin requests.
- Implemented health check endpoint for service monitoring.
- Enhanced existing CSV and Excel sample files with additional fields.
- Introduced a region selection component and dynamic filter form in the shared filter-builder package.
</commit_message>
<xml_diff>
--- a/services/file-import-service/samples/calls.xlsx
+++ b/services/file-import-service/samples/calls.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,7 +434,12 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>通话时长(秒)</t>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>times</t>
         </is>
       </c>
     </row>
@@ -457,6 +462,9 @@
       <c r="D2" t="n">
         <v>85</v>
       </c>
+      <c r="E2" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -477,6 +485,9 @@
       <c r="D3" t="n">
         <v>42</v>
       </c>
+      <c r="E3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -496,6 +507,9 @@
       </c>
       <c r="D4" t="n">
         <v>120</v>
+      </c>
+      <c r="E4" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>